<commit_message>
Add link column to excel and update script
</commit_message>
<xml_diff>
--- a/hanzicraft_dashboard.xlsx
+++ b/hanzicraft_dashboard.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B251"/>
+  <dimension ref="A1:C251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,11 @@
           <t>Chữ Hán</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -437,6 +442,11 @@
           <t>的</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9A%84</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -447,6 +457,11 @@
           <t>一</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%80</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -457,6 +472,11 @@
           <t>是</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%98%AF</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -467,6 +487,11 @@
           <t>不</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%8D</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -477,6 +502,11 @@
           <t>了</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%86</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -487,6 +517,11 @@
           <t>在</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9C%A8</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -497,6 +532,11 @@
           <t>人</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%BA</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -507,6 +547,11 @@
           <t>有</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%89</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -517,6 +562,11 @@
           <t>我</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%88%91</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -527,6 +577,11 @@
           <t>他</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%96</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -537,6 +592,11 @@
           <t>这</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%99</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -547,6 +607,11 @@
           <t>个</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%AA</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -557,6 +622,11 @@
           <t>们</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%AC</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -567,6 +637,11 @@
           <t>中</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%AD</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -577,6 +652,11 @@
           <t>来</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%A5</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -587,6 +667,11 @@
           <t>上</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%8A</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -597,6 +682,11 @@
           <t>大</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%A7</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -607,6 +697,11 @@
           <t>为</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%BA</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -617,6 +712,11 @@
           <t>和</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%92%8C</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -627,6 +727,11 @@
           <t>国</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9B%BD</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -637,6 +742,11 @@
           <t>地</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9C%B0</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -647,6 +757,11 @@
           <t>到</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%B0</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -657,6 +772,11 @@
           <t>以</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%A5</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -667,6 +787,11 @@
           <t>说</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%B4</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -677,6 +802,11 @@
           <t>时</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%97%B6</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -687,6 +817,11 @@
           <t>要</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A6%81</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -697,6 +832,11 @@
           <t>就</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%B1</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -707,6 +847,11 @@
           <t>出</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%87%BA</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -717,6 +862,11 @@
           <t>会</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BC%9A</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -727,6 +877,11 @@
           <t>可</t>
         </is>
       </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%AF</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -737,6 +892,11 @@
           <t>也</t>
         </is>
       </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%9F</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -747,6 +907,11 @@
           <t>你</t>
         </is>
       </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%A0</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -757,6 +922,11 @@
           <t>对</t>
         </is>
       </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AF%B9</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -767,6 +937,11 @@
           <t>生</t>
         </is>
       </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%94%9F</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -777,6 +952,11 @@
           <t>能</t>
         </is>
       </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%83%BD</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -787,6 +967,11 @@
           <t>而</t>
         </is>
       </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%80%8C</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -797,6 +982,11 @@
           <t>子</t>
         </is>
       </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AD%90</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -807,6 +997,11 @@
           <t>那</t>
         </is>
       </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%82%A3</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -817,6 +1012,11 @@
           <t>得</t>
         </is>
       </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BE%97</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -827,6 +1027,11 @@
           <t>于</t>
         </is>
       </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%8E</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -837,6 +1042,11 @@
           <t>着</t>
         </is>
       </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9D%80</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -847,6 +1057,11 @@
           <t>下</t>
         </is>
       </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%8B</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -857,6 +1072,11 @@
           <t>自</t>
         </is>
       </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%87%AA</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -867,6 +1087,11 @@
           <t>之</t>
         </is>
       </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%8B</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -877,6 +1102,11 @@
           <t>年</t>
         </is>
       </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B9%B4</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -887,6 +1117,11 @@
           <t>过</t>
         </is>
       </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%87</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -897,6 +1132,11 @@
           <t>发</t>
         </is>
       </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%91</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -907,6 +1147,11 @@
           <t>后</t>
         </is>
       </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%8E</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -917,6 +1162,11 @@
           <t>作</t>
         </is>
       </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%9C</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -927,6 +1177,11 @@
           <t>里</t>
         </is>
       </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%87%8C</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -937,6 +1192,11 @@
           <t>用</t>
         </is>
       </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%94%A8</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -947,6 +1207,11 @@
           <t>道</t>
         </is>
       </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%81%93</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -957,6 +1222,11 @@
           <t>行</t>
         </is>
       </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A1%8C</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -967,6 +1237,11 @@
           <t>所</t>
         </is>
       </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%80</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -977,6 +1252,11 @@
           <t>然</t>
         </is>
       </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%84%B6</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -987,6 +1267,11 @@
           <t>家</t>
         </is>
       </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%B6</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -997,6 +1282,11 @@
           <t>种</t>
         </is>
       </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A7%8D</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1007,6 +1297,11 @@
           <t>事</t>
         </is>
       </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%8B</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1017,6 +1312,11 @@
           <t>成</t>
         </is>
       </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%88%90</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1027,6 +1327,11 @@
           <t>方</t>
         </is>
       </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%96%B9</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1037,6 +1342,11 @@
           <t>多</t>
         </is>
       </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%9A</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1047,6 +1357,11 @@
           <t>经</t>
         </is>
       </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%8F</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1057,6 +1372,11 @@
           <t>么</t>
         </is>
       </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%88</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1067,6 +1387,11 @@
           <t>去</t>
         </is>
       </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%BB</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1077,6 +1402,11 @@
           <t>法</t>
         </is>
       </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B3%95</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1087,6 +1417,11 @@
           <t>学</t>
         </is>
       </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AD%A6</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1097,6 +1432,11 @@
           <t>如</t>
         </is>
       </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A6%82</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1107,6 +1447,11 @@
           <t>都</t>
         </is>
       </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%83%BD</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1117,6 +1462,11 @@
           <t>同</t>
         </is>
       </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%8C</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1127,6 +1477,11 @@
           <t>现</t>
         </is>
       </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%8E%B0</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1137,6 +1492,11 @@
           <t>当</t>
         </is>
       </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BD%93</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -1147,6 +1507,11 @@
           <t>没</t>
         </is>
       </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B2%A1</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1157,6 +1522,11 @@
           <t>动</t>
         </is>
       </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%A8</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -1167,6 +1537,11 @@
           <t>面</t>
         </is>
       </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%9D%A2</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -1177,6 +1552,11 @@
           <t>起</t>
         </is>
       </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%B7</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -1187,6 +1567,11 @@
           <t>看</t>
         </is>
       </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9C%8B</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -1197,6 +1582,11 @@
           <t>定</t>
         </is>
       </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%9A</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -1207,6 +1597,11 @@
           <t>天</t>
         </is>
       </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%A9</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -1217,6 +1612,11 @@
           <t>分</t>
         </is>
       </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%86</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -1227,6 +1627,11 @@
           <t>还</t>
         </is>
       </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%98</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -1237,6 +1642,11 @@
           <t>进</t>
         </is>
       </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BF%9B</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -1247,6 +1657,11 @@
           <t>好</t>
         </is>
       </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A5%BD</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -1257,6 +1672,11 @@
           <t>小</t>
         </is>
       </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%8F</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -1267,6 +1687,11 @@
           <t>部</t>
         </is>
       </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%83%A8</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -1277,6 +1702,11 @@
           <t>其</t>
         </is>
       </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%B6</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -1287,6 +1717,11 @@
           <t>些</t>
         </is>
       </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%9B</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -1297,6 +1732,11 @@
           <t>主</t>
         </is>
       </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%BB</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -1307,6 +1747,11 @@
           <t>样</t>
         </is>
       </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%A0%B7</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -1317,6 +1762,11 @@
           <t>理</t>
         </is>
       </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%90%86</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -1327,6 +1777,11 @@
           <t>心</t>
         </is>
       </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BF%83</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -1337,6 +1792,11 @@
           <t>她</t>
         </is>
       </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A5%B9</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -1347,6 +1807,11 @@
           <t>本</t>
         </is>
       </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%AC</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -1357,6 +1822,11 @@
           <t>前</t>
         </is>
       </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%89%8D</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -1367,6 +1837,11 @@
           <t>开</t>
         </is>
       </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BC%80</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -1377,6 +1852,11 @@
           <t>但</t>
         </is>
       </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%86</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -1387,6 +1867,11 @@
           <t>因</t>
         </is>
       </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9B%A0</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -1397,6 +1882,11 @@
           <t>只</t>
         </is>
       </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%AA</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -1407,6 +1897,11 @@
           <t>从</t>
         </is>
       </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%8E</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -1417,6 +1912,11 @@
           <t>想</t>
         </is>
       </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%83%B3</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -1427,6 +1927,11 @@
           <t>实</t>
         </is>
       </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%9E</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -1437,6 +1942,11 @@
           <t>日</t>
         </is>
       </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%97%A5</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -1447,6 +1957,11 @@
           <t>军</t>
         </is>
       </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%9B</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -1457,6 +1972,11 @@
           <t>者</t>
         </is>
       </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%80%85</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -1467,6 +1987,11 @@
           <t>意</t>
         </is>
       </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%84%8F</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -1477,6 +2002,11 @@
           <t>无</t>
         </is>
       </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%97%A0</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -1487,6 +2017,11 @@
           <t>力</t>
         </is>
       </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%9B</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -1497,6 +2032,11 @@
           <t>它</t>
         </is>
       </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%83</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -1507,6 +2047,11 @@
           <t>与</t>
         </is>
       </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%8E</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -1517,6 +2062,11 @@
           <t>长</t>
         </is>
       </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%95%BF</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -1527,6 +2077,11 @@
           <t>把</t>
         </is>
       </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%8A</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -1537,6 +2092,11 @@
           <t>机</t>
         </is>
       </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%BA</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -1547,6 +2107,11 @@
           <t>十</t>
         </is>
       </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8D%81</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -1557,6 +2122,11 @@
           <t>民</t>
         </is>
       </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B0%91</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -1567,6 +2137,11 @@
           <t>第</t>
         </is>
       </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AC%AC</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -1577,6 +2152,11 @@
           <t>公</t>
         </is>
       </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%AC</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -1587,6 +2167,11 @@
           <t>此</t>
         </is>
       </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AD%A4</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -1597,6 +2182,11 @@
           <t>已</t>
         </is>
       </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B7%B2</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -1607,6 +2197,11 @@
           <t>工</t>
         </is>
       </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B7%A5</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -1617,6 +2212,11 @@
           <t>使</t>
         </is>
       </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%BF</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -1627,6 +2227,11 @@
           <t>情</t>
         </is>
       </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%83%85</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -1637,6 +2242,11 @@
           <t>明</t>
         </is>
       </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%98%8E</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -1647,6 +2257,11 @@
           <t>性</t>
         </is>
       </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%A7</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -1657,6 +2272,11 @@
           <t>知</t>
         </is>
       </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9F%A5</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -1667,6 +2287,11 @@
           <t>全</t>
         </is>
       </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%A8</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -1677,6 +2302,11 @@
           <t>三</t>
         </is>
       </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%89</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -1687,6 +2317,11 @@
           <t>又</t>
         </is>
       </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%88</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -1697,6 +2332,11 @@
           <t>关</t>
         </is>
       </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%B3</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -1707,6 +2347,11 @@
           <t>点</t>
         </is>
       </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%82%B9</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -1717,6 +2362,11 @@
           <t>正</t>
         </is>
       </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AD%A3</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -1727,6 +2377,11 @@
           <t>业</t>
         </is>
       </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%9A</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -1737,6 +2392,11 @@
           <t>外</t>
         </is>
       </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%96</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -1747,6 +2407,11 @@
           <t>将</t>
         </is>
       </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%86</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -1757,6 +2422,11 @@
           <t>两</t>
         </is>
       </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%A4</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -1767,6 +2437,11 @@
           <t>高</t>
         </is>
       </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%AB%98</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -1777,6 +2452,11 @@
           <t>间</t>
         </is>
       </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%97%B4</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -1787,6 +2467,11 @@
           <t>由</t>
         </is>
       </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%94%B1</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -1797,6 +2482,11 @@
           <t>问</t>
         </is>
       </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%97%AE</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -1807,6 +2497,11 @@
           <t>很</t>
         </is>
       </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BE%88</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -1817,6 +2512,11 @@
           <t>最</t>
         </is>
       </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%80</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -1827,6 +2527,11 @@
           <t>重</t>
         </is>
       </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%87%8D</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -1837,6 +2542,11 @@
           <t>并</t>
         </is>
       </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B9%B6</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -1847,6 +2557,11 @@
           <t>物</t>
         </is>
       </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%89%A9</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -1857,6 +2572,11 @@
           <t>手</t>
         </is>
       </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%8B</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -1867,6 +2587,11 @@
           <t>应</t>
         </is>
       </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%94</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -1877,6 +2602,11 @@
           <t>战</t>
         </is>
       </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%88%98</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -1887,6 +2617,11 @@
           <t>向</t>
         </is>
       </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%91</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -1897,6 +2632,11 @@
           <t>头</t>
         </is>
       </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%B4</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -1907,6 +2647,11 @@
           <t>文</t>
         </is>
       </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%96%87</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -1917,6 +2662,11 @@
           <t>体</t>
         </is>
       </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%93</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -1927,6 +2677,11 @@
           <t>政</t>
         </is>
       </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%94%BF</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -1937,6 +2692,11 @@
           <t>美</t>
         </is>
       </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BE%8E</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -1947,6 +2707,11 @@
           <t>相</t>
         </is>
       </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%B8</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -1957,6 +2722,11 @@
           <t>见</t>
         </is>
       </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A7%81</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -1967,6 +2737,11 @@
           <t>被</t>
         </is>
       </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A2%AB</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -1977,6 +2752,11 @@
           <t>利</t>
         </is>
       </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%A9</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -1987,6 +2767,11 @@
           <t>什</t>
         </is>
       </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%80</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -1997,6 +2782,11 @@
           <t>二</t>
         </is>
       </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%8C</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -2007,6 +2797,11 @@
           <t>等</t>
         </is>
       </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AD%89</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -2017,6 +2812,11 @@
           <t>产</t>
         </is>
       </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BA%A7</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -2027,6 +2827,11 @@
           <t>或</t>
         </is>
       </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%88%96</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -2037,6 +2842,11 @@
           <t>新</t>
         </is>
       </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%96%B0</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -2047,6 +2857,11 @@
           <t>己</t>
         </is>
       </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B7%B1</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -2057,6 +2872,11 @@
           <t>制</t>
         </is>
       </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%B6</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -2067,6 +2887,11 @@
           <t>身</t>
         </is>
       </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%BA%AB</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -2077,6 +2902,11 @@
           <t>果</t>
         </is>
       </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9E%9C</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -2087,6 +2917,11 @@
           <t>加</t>
         </is>
       </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%A0</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -2097,6 +2932,11 @@
           <t>西</t>
         </is>
       </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A5%BF</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -2107,6 +2947,11 @@
           <t>斯</t>
         </is>
       </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%96%AF</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -2117,6 +2962,11 @@
           <t>月</t>
         </is>
       </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9C%88</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -2127,6 +2977,11 @@
           <t>话</t>
         </is>
       </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AF%9D</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -2137,6 +2992,11 @@
           <t>合</t>
         </is>
       </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%88</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -2147,6 +3007,11 @@
           <t>回</t>
         </is>
       </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9B%9E</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -2157,6 +3022,11 @@
           <t>特</t>
         </is>
       </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%89%B9</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -2167,6 +3037,11 @@
           <t>代</t>
         </is>
       </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%A3</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -2177,6 +3052,11 @@
           <t>内</t>
         </is>
       </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%85</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -2187,6 +3067,11 @@
           <t>信</t>
         </is>
       </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BF%A1</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -2197,6 +3082,11 @@
           <t>表</t>
         </is>
       </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A1%A8</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -2207,6 +3097,11 @@
           <t>化</t>
         </is>
       </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8C%96</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -2217,6 +3112,11 @@
           <t>老</t>
         </is>
       </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%80%81</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -2227,6 +3127,11 @@
           <t>给</t>
         </is>
       </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%99</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -2237,6 +3142,11 @@
           <t>世</t>
         </is>
       </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%96</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -2247,6 +3157,11 @@
           <t>位</t>
         </is>
       </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%8D</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -2257,6 +3172,11 @@
           <t>次</t>
         </is>
       </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AC%A1</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -2267,6 +3187,11 @@
           <t>度</t>
         </is>
       </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BA%A6</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -2277,6 +3202,11 @@
           <t>门</t>
         </is>
       </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%97%A8</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -2287,6 +3217,11 @@
           <t>任</t>
         </is>
       </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%BB</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -2297,6 +3232,11 @@
           <t>常</t>
         </is>
       </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B8%B8</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -2307,6 +3247,11 @@
           <t>先</t>
         </is>
       </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%88</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -2317,6 +3262,11 @@
           <t>海</t>
         </is>
       </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B5%B7</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -2327,6 +3277,11 @@
           <t>通</t>
         </is>
       </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%80%9A</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -2337,6 +3292,11 @@
           <t>教</t>
         </is>
       </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%99</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -2347,6 +3307,11 @@
           <t>儿</t>
         </is>
       </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%84%BF</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -2357,6 +3322,11 @@
           <t>原</t>
         </is>
       </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8E%9F</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -2367,6 +3337,11 @@
           <t>东</t>
         </is>
       </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B8%9C</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -2377,6 +3352,11 @@
           <t>声</t>
         </is>
       </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A3%B0</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -2387,6 +3367,11 @@
           <t>提</t>
         </is>
       </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8F%90</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -2397,6 +3382,11 @@
           <t>立</t>
         </is>
       </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%AB%8B</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -2407,6 +3397,11 @@
           <t>及</t>
         </is>
       </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%8A</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -2417,6 +3412,11 @@
           <t>比</t>
         </is>
       </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%AF%94</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -2427,6 +3427,11 @@
           <t>员</t>
         </is>
       </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%91%98</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -2437,6 +3442,11 @@
           <t>解</t>
         </is>
       </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%A7%A3</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -2447,6 +3457,11 @@
           <t>水</t>
         </is>
       </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B0%B4</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -2457,6 +3472,11 @@
           <t>名</t>
         </is>
       </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%8D</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -2467,6 +3487,11 @@
           <t>真</t>
         </is>
       </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9C%9F</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -2477,6 +3502,11 @@
           <t>论</t>
         </is>
       </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%BA</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -2487,6 +3517,11 @@
           <t>处</t>
         </is>
       </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%84</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -2497,6 +3532,11 @@
           <t>走</t>
         </is>
       </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%B5%B0</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -2507,6 +3547,11 @@
           <t>义</t>
         </is>
       </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%B9%89</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -2517,6 +3562,11 @@
           <t>各</t>
         </is>
       </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%90%84</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -2527,6 +3577,11 @@
           <t>入</t>
         </is>
       </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%85%A5</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -2537,6 +3592,11 @@
           <t>几</t>
         </is>
       </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%87%A0</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -2547,6 +3607,11 @@
           <t>口</t>
         </is>
       </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%A3</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -2557,6 +3622,11 @@
           <t>认</t>
         </is>
       </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E8%AE%A4</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -2567,6 +3637,11 @@
           <t>条</t>
         </is>
       </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9D%A1</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -2577,6 +3652,11 @@
           <t>平</t>
         </is>
       </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B9%B3</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -2587,6 +3667,11 @@
           <t>系</t>
         </is>
       </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%B3%BB</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -2597,6 +3682,11 @@
           <t>气</t>
         </is>
       </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B0%94</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -2607,6 +3697,11 @@
           <t>题</t>
         </is>
       </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%A2%98</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -2617,6 +3712,11 @@
           <t>活</t>
         </is>
       </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%B4%BB</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -2627,6 +3727,11 @@
           <t>尔</t>
         </is>
       </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%94</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -2637,6 +3742,11 @@
           <t>更</t>
         </is>
       </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%9B%B4</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -2647,6 +3757,11 @@
           <t>别</t>
         </is>
       </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%88%AB</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -2657,6 +3772,11 @@
           <t>打</t>
         </is>
       </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%93</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -2667,6 +3787,11 @@
           <t>女</t>
         </is>
       </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A5%B3</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -2677,6 +3802,11 @@
           <t>变</t>
         </is>
       </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%98</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -2687,6 +3817,11 @@
           <t>四</t>
         </is>
       </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9B%9B</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -2697,6 +3832,11 @@
           <t>神</t>
         </is>
       </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%A5%9E</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -2707,6 +3847,11 @@
           <t>总</t>
         </is>
       </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%80%BB</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -2717,6 +3862,11 @@
           <t>何</t>
         </is>
       </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BD%95</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -2727,6 +3877,11 @@
           <t>电</t>
         </is>
       </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%94%B5</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -2737,6 +3892,11 @@
           <t>数</t>
         </is>
       </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%95%B0</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -2747,6 +3907,11 @@
           <t>安</t>
         </is>
       </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%AE%89</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -2757,6 +3922,11 @@
           <t>少</t>
         </is>
       </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%B0%91</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -2767,6 +3937,11 @@
           <t>报</t>
         </is>
       </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8A%A5</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -2777,6 +3952,11 @@
           <t>才</t>
         </is>
       </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%89%8D</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -2787,6 +3967,11 @@
           <t>结</t>
         </is>
       </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%BB%93</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -2797,6 +3982,11 @@
           <t>反</t>
         </is>
       </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%8D</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -2807,6 +3997,11 @@
           <t>受</t>
         </is>
       </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8F%97</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -2817,6 +4012,11 @@
           <t>目</t>
         </is>
       </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E7%9B%AE</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -2827,6 +4027,11 @@
           <t>太</t>
         </is>
       </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%A4%AA</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -2837,6 +4042,11 @@
           <t>量</t>
         </is>
       </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E9%87%8F</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -2847,6 +4057,11 @@
           <t>再</t>
         </is>
       </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%86%8D</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -2857,6 +4072,11 @@
           <t>感</t>
         </is>
       </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%84%9F</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -2867,6 +4087,11 @@
           <t>建</t>
         </is>
       </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BB%BA</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -2877,6 +4102,11 @@
           <t>务</t>
         </is>
       </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%8A%A1</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -2887,6 +4117,11 @@
           <t>做</t>
         </is>
       </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%81%9A</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -2897,6 +4132,11 @@
           <t>接</t>
         </is>
       </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E6%8E%A5</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -2907,6 +4147,11 @@
           <t>必</t>
         </is>
       </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%BF%85</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -2917,6 +4162,11 @@
           <t>场</t>
         </is>
       </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E5%9C%BA</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -2925,6 +4175,11 @@
       <c r="B251" t="inlineStr">
         <is>
           <t>件</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>https://hanzicraft.com/dashboard/character/%E4%BB%B6</t>
         </is>
       </c>
     </row>

</xml_diff>